<commit_message>
heterogeneous xylem pressure introduced, remain to impact back the properties
</commit_message>
<xml_diff>
--- a/simulations/inputs/Scenarios_24_11_10.xlsx
+++ b/simulations/inputs/Scenarios_24_11_10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\sshfs\torisuten@192.168.12.9\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8242209-1EDC-4138-96AF-EAA2E98D8286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C097F1-00FC-4FCE-AF4F-5387B83E0989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28785" yWindow="-21435" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -2641,48 +2641,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
     <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
     <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
     <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
     <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
     <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Avertissement" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Calcul" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Cellule liée" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Entrée" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Insatisfaisant" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Neutre" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Satisfaisant" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Sortie" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texte explicatif" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Titre" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Titre 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Titre 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Titre 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Titre 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Vérification" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2961,17 +2961,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M234"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" style="1" customWidth="1"/>
     <col min="2" max="4" width="15" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" style="37" customWidth="1"/>
-    <col min="8" max="13" width="39.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.21875" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" style="37" customWidth="1"/>
+    <col min="8" max="13" width="39.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>469</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>532</v>
       </c>
@@ -3047,7 +3047,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>472</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>484</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>483</v>
       </c>
@@ -3161,7 +3161,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>490</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>485</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>537</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -3313,7 +3313,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="74" t="s">
         <v>444</v>
       </c>
@@ -3389,7 +3389,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>4</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>5</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>4.1666666999999998E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>20</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>4.1666666999999998E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>1</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>448</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>6</v>
       </c>
@@ -3617,7 +3617,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>7</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>5.0000000000000001E-9</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
@@ -3693,7 +3693,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>461</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>462</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>465</v>
       </c>
@@ -3807,7 +3807,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>467</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>86400</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>10</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>11</v>
       </c>
@@ -3921,7 +3921,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>363</v>
       </c>
@@ -3959,7 +3959,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>365</v>
       </c>
@@ -3997,7 +3997,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>377</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>376</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>375</v>
       </c>
@@ -4111,7 +4111,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>12</v>
       </c>
@@ -4149,7 +4149,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>13</v>
       </c>
@@ -4187,7 +4187,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>14</v>
       </c>
@@ -4225,7 +4225,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>9</v>
       </c>
@@ -4263,7 +4263,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>454</v>
       </c>
@@ -4301,7 +4301,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
         <v>21</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="13" t="s">
         <v>22</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
         <v>23</v>
       </c>
@@ -4415,7 +4415,7 @@
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
         <v>24</v>
       </c>
@@ -4453,7 +4453,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
         <v>25</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
         <v>26</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>27</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
         <v>28</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="13" t="s">
         <v>29</v>
       </c>
@@ -4643,7 +4643,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="13" t="s">
         <v>30</v>
       </c>
@@ -4681,7 +4681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="13" t="s">
         <v>31</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="13" t="s">
         <v>32</v>
       </c>
@@ -4757,7 +4757,7 @@
         <v>-0.1</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="13" t="s">
         <v>33</v>
       </c>
@@ -4795,7 +4795,7 @@
         <v>-0.2</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="13" t="s">
         <v>34</v>
       </c>
@@ -4833,7 +4833,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
         <v>35</v>
       </c>
@@ -4871,7 +4871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" s="13" t="s">
         <v>434</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>435</v>
       </c>
@@ -4947,7 +4947,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" s="13" t="s">
         <v>457</v>
       </c>
@@ -4985,7 +4985,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" s="13" t="s">
         <v>15</v>
       </c>
@@ -5023,7 +5023,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
         <v>16</v>
       </c>
@@ -5061,7 +5061,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
         <v>17</v>
       </c>
@@ -5099,7 +5099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>18</v>
       </c>
@@ -5137,7 +5137,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>19</v>
       </c>
@@ -5175,7 +5175,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" s="15" t="s">
         <v>36</v>
       </c>
@@ -5213,7 +5213,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" s="15" t="s">
         <v>380</v>
       </c>
@@ -5251,7 +5251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" s="15" t="s">
         <v>37</v>
       </c>
@@ -5289,7 +5289,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="15" t="s">
         <v>38</v>
       </c>
@@ -5327,7 +5327,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="17" t="s">
         <v>39</v>
       </c>
@@ -5365,7 +5365,7 @@
         <v>6.9999999999999999E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="17" t="s">
         <v>40</v>
       </c>
@@ -5403,7 +5403,7 @@
         <v>1.22E-4</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" s="17" t="s">
         <v>207</v>
       </c>
@@ -5441,7 +5441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
         <v>41</v>
       </c>
@@ -5479,7 +5479,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" s="17" t="s">
         <v>406</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" s="17" t="s">
         <v>91</v>
       </c>
@@ -5555,7 +5555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" s="17" t="s">
         <v>408</v>
       </c>
@@ -5593,7 +5593,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" s="17" t="s">
         <v>42</v>
       </c>
@@ -5631,7 +5631,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" s="17" t="s">
         <v>208</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>1453890.8941884842</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="17" t="s">
         <v>43</v>
       </c>
@@ -5707,7 +5707,7 @@
         <v>1.3888888888888888E-5</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" s="17" t="s">
         <v>44</v>
       </c>
@@ -5745,7 +5745,7 @@
         <v>6.5011574074074071E-4</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" s="17" t="s">
         <v>45</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>4.7400000000000003E-3</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" s="17" t="s">
         <v>46</v>
       </c>
@@ -5821,7 +5821,7 @@
         <v>282528</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" s="17" t="s">
         <v>47</v>
       </c>
@@ -5859,7 +5859,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" s="17" t="s">
         <v>48</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" s="17" t="s">
         <v>49</v>
       </c>
@@ -5935,7 +5935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" s="33" t="s">
         <v>50</v>
       </c>
@@ -5973,7 +5973,7 @@
         <v>745476480000</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" s="33" t="s">
         <v>205</v>
       </c>
@@ -6011,7 +6011,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" s="33" t="s">
         <v>414</v>
       </c>
@@ -6049,7 +6049,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" s="33" t="s">
         <v>400</v>
       </c>
@@ -6087,7 +6087,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" s="33" t="s">
         <v>410</v>
       </c>
@@ -6125,7 +6125,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" s="33" t="s">
         <v>401</v>
       </c>
@@ -6163,7 +6163,7 @@
         <v>60479.999999999993</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" s="33" t="s">
         <v>411</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" s="33" t="s">
         <v>402</v>
       </c>
@@ -6239,7 +6239,7 @@
         <v>518400</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" s="33" t="s">
         <v>412</v>
       </c>
@@ -6277,7 +6277,7 @@
         <v>5184000</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" s="17" t="s">
         <v>51</v>
       </c>
@@ -6315,7 +6315,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" s="17" t="s">
         <v>52</v>
       </c>
@@ -6353,7 +6353,7 @@
         <v>140000</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" s="17" t="s">
         <v>53</v>
       </c>
@@ -6391,7 +6391,7 @@
         <v>3.6636136999999999E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" s="17" t="s">
         <v>54</v>
       </c>
@@ -6429,7 +6429,7 @@
         <v>4.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" s="17" t="s">
         <v>55</v>
       </c>
@@ -6467,7 +6467,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" s="19" t="s">
         <v>214</v>
       </c>
@@ -6505,7 +6505,7 @@
         <v>6.0000000000000002E-6</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" s="19" t="s">
         <v>215</v>
       </c>
@@ -6543,7 +6543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" s="19" t="s">
         <v>216</v>
       </c>
@@ -6581,7 +6581,7 @@
         <v>374999999.99999994</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" s="19" t="s">
         <v>217</v>
       </c>
@@ -6619,7 +6619,7 @@
         <v>3.7037037037037038E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" s="19" t="s">
         <v>218</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>165600</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" s="13" t="s">
         <v>60</v>
       </c>
@@ -6695,7 +6695,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" s="13" t="s">
         <v>209</v>
       </c>
@@ -6733,7 +6733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" s="13" t="s">
         <v>59</v>
       </c>
@@ -6771,7 +6771,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" s="23" t="s">
         <v>65</v>
       </c>
@@ -6809,7 +6809,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" s="23" t="s">
         <v>367</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" s="23" t="s">
         <v>368</v>
       </c>
@@ -6885,7 +6885,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" s="23" t="s">
         <v>369</v>
       </c>
@@ -6923,7 +6923,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" s="23" t="s">
         <v>501</v>
       </c>
@@ -6961,7 +6961,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" s="23" t="s">
         <v>385</v>
       </c>
@@ -6999,7 +6999,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" s="23" t="s">
         <v>502</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" s="23" t="s">
         <v>503</v>
       </c>
@@ -7083,7 +7083,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" s="23" t="s">
         <v>504</v>
       </c>
@@ -7125,7 +7125,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" s="23" t="s">
         <v>505</v>
       </c>
@@ -7167,7 +7167,7 @@
         <v>1470</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" s="23" t="s">
         <v>387</v>
       </c>
@@ -7205,7 +7205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" s="23" t="s">
         <v>389</v>
       </c>
@@ -7243,7 +7243,7 @@
         <v>1589759.9999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" s="23" t="s">
         <v>391</v>
       </c>
@@ -7281,7 +7281,7 @@
         <v>6171428.5714285718</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" s="23" t="s">
         <v>393</v>
       </c>
@@ -7319,7 +7319,7 @@
         <v>6171428.5714285718</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" s="23" t="s">
         <v>421</v>
       </c>
@@ -7357,7 +7357,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="116" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="23" t="s">
         <v>423</v>
       </c>
@@ -7399,7 +7399,7 @@
         <v>28080</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" s="23" t="s">
         <v>425</v>
       </c>
@@ -7441,7 +7441,7 @@
         <v>0.11100000000000002</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" s="23" t="s">
         <v>498</v>
       </c>
@@ -7479,7 +7479,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="119" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="23" t="s">
         <v>499</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>459648</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A120" s="23" t="s">
         <v>500</v>
       </c>
@@ -7563,7 +7563,7 @@
         <v>0.13875000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A121" s="23" t="s">
         <v>395</v>
       </c>
@@ -7601,7 +7601,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A122" s="23" t="s">
         <v>397</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>43200</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A123" s="13" t="s">
         <v>61</v>
       </c>
@@ -7677,7 +7677,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A124" s="13" t="s">
         <v>62</v>
       </c>
@@ -7716,7 +7716,7 @@
         <v>2.0833333333333335E-4</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A125" s="13" t="s">
         <v>63</v>
       </c>
@@ -7754,7 +7754,7 @@
         <v>5.7899999999999998E-7</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A126" s="13" t="s">
         <v>64</v>
       </c>
@@ -7792,7 +7792,7 @@
         <v>2.0833333333333335E-4</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A127" s="13" t="s">
         <v>450</v>
       </c>
@@ -7830,7 +7830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A128" s="13" t="s">
         <v>452</v>
       </c>
@@ -7868,7 +7868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A129" s="68" t="s">
         <v>441</v>
       </c>
@@ -7909,7 +7909,7 @@
         <v>5.9999999999999997E-7</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A130" s="68" t="s">
         <v>67</v>
       </c>
@@ -7950,7 +7950,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A131" s="68" t="s">
         <v>446</v>
       </c>
@@ -7988,7 +7988,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A132" s="21" t="s">
         <v>66</v>
       </c>
@@ -8026,7 +8026,7 @@
         <v>5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A133" s="21" t="s">
         <v>438</v>
       </c>
@@ -8064,7 +8064,7 @@
         <v>4.9999999999999999E-13</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A134" s="21" t="s">
         <v>229</v>
       </c>
@@ -8102,7 +8102,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A135" s="21" t="s">
         <v>230</v>
       </c>
@@ -8140,7 +8140,7 @@
         <v>-0.04</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A136" s="21" t="s">
         <v>231</v>
       </c>
@@ -8178,7 +8178,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A137" s="21" t="s">
         <v>232</v>
       </c>
@@ -8216,7 +8216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A138" s="21" t="s">
         <v>68</v>
       </c>
@@ -8254,7 +8254,7 @@
         <v>1.9999999999999999E-7</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A139" s="21" t="s">
         <v>233</v>
       </c>
@@ -8292,7 +8292,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A140" s="21" t="s">
         <v>234</v>
       </c>
@@ -8330,7 +8330,7 @@
         <v>-0.04</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A141" s="21" t="s">
         <v>235</v>
       </c>
@@ -8368,7 +8368,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A142" s="21" t="s">
         <v>236</v>
       </c>
@@ -8406,7 +8406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A143" s="21" t="s">
         <v>69</v>
       </c>
@@ -8444,7 +8444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A144" s="72" t="s">
         <v>70</v>
       </c>
@@ -8482,7 +8482,7 @@
         <v>5.0000000000000004E-6</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A145" s="23" t="s">
         <v>56</v>
       </c>
@@ -8520,7 +8520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A146" s="23" t="s">
         <v>57</v>
       </c>
@@ -8558,7 +8558,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A147" s="23" t="s">
         <v>58</v>
       </c>
@@ -8596,7 +8596,7 @@
         <v>3.9999999999999998E-6</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A148" s="23" t="s">
         <v>71</v>
       </c>
@@ -8634,7 +8634,7 @@
         <v>3.7699999999999999E-10</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A149" s="23" t="s">
         <v>237</v>
       </c>
@@ -8672,7 +8672,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A150" s="23" t="s">
         <v>238</v>
       </c>
@@ -8710,7 +8710,7 @@
         <v>-0.06</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A151" s="23" t="s">
         <v>239</v>
       </c>
@@ -8748,7 +8748,7 @@
         <v>0.89100000000000001</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A152" s="23" t="s">
         <v>240</v>
       </c>
@@ -8786,7 +8786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A153" s="23" t="s">
         <v>72</v>
       </c>
@@ -8824,7 +8824,7 @@
         <v>4.0000000000000003E-5</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A154" s="13" t="s">
         <v>73</v>
       </c>
@@ -8862,7 +8862,7 @@
         <v>5.8333333333333335E-9</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A155" s="13" t="s">
         <v>241</v>
       </c>
@@ -8900,7 +8900,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A156" s="13" t="s">
         <v>242</v>
       </c>
@@ -8938,7 +8938,7 @@
         <v>-0.06</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A157" s="13" t="s">
         <v>243</v>
       </c>
@@ -8976,7 +8976,7 @@
         <v>0.89100000000000001</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A158" s="13" t="s">
         <v>244</v>
       </c>
@@ -9014,7 +9014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A159" s="13" t="s">
         <v>74</v>
       </c>
@@ -9052,7 +9052,7 @@
         <v>4.0000000000000003E-5</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A160" s="9" t="s">
         <v>75</v>
       </c>
@@ -9090,7 +9090,7 @@
         <v>4.0000000000000001E-8</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A161" s="9" t="s">
         <v>219</v>
       </c>
@@ -9128,7 +9128,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A162" s="9" t="s">
         <v>220</v>
       </c>
@@ -9166,7 +9166,7 @@
         <v>-4.4200000000000003E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A163" s="9" t="s">
         <v>221</v>
       </c>
@@ -9204,7 +9204,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A164" s="9" t="s">
         <v>222</v>
       </c>
@@ -9242,7 +9242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A165" s="9" t="s">
         <v>76</v>
       </c>
@@ -9280,7 +9280,7 @@
         <v>2.7799999999999998E-4</v>
       </c>
     </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A166" s="25" t="s">
         <v>78</v>
       </c>
@@ -9318,7 +9318,7 @@
         <v>2.4999999999999998E-12</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A167" s="25" t="s">
         <v>246</v>
       </c>
@@ -9356,7 +9356,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A168" s="25" t="s">
         <v>247</v>
       </c>
@@ -9394,7 +9394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A169" s="25" t="s">
         <v>248</v>
       </c>
@@ -9432,7 +9432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A170" s="25" t="s">
         <v>249</v>
       </c>
@@ -9470,7 +9470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A171" s="25" t="s">
         <v>79</v>
       </c>
@@ -9508,7 +9508,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A172" s="31" t="s">
         <v>80</v>
       </c>
@@ -9546,7 +9546,7 @@
         <v>2.0000000000000001E-9</v>
       </c>
     </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A173" s="31" t="s">
         <v>250</v>
       </c>
@@ -9584,7 +9584,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A174" s="31" t="s">
         <v>251</v>
       </c>
@@ -9622,7 +9622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A175" s="31" t="s">
         <v>252</v>
       </c>
@@ -9660,7 +9660,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A176" s="31" t="s">
         <v>253</v>
       </c>
@@ -9698,7 +9698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A177" s="31" t="s">
         <v>81</v>
       </c>
@@ -9736,7 +9736,7 @@
         <v>1.6666666666666666E-4</v>
       </c>
     </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A178" s="11" t="s">
         <v>254</v>
       </c>
@@ -9774,7 +9774,7 @@
         <v>1E-8</v>
       </c>
     </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A179" s="11" t="s">
         <v>255</v>
       </c>
@@ -9812,7 +9812,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A180" s="11" t="s">
         <v>256</v>
       </c>
@@ -9850,7 +9850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A181" s="11" t="s">
         <v>257</v>
       </c>
@@ -9888,7 +9888,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A182" s="11" t="s">
         <v>258</v>
       </c>
@@ -9926,7 +9926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A183" s="11" t="s">
         <v>259</v>
       </c>
@@ -9964,7 +9964,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A184" s="11" t="s">
         <v>260</v>
       </c>
@@ -10002,7 +10002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A185" s="27" t="s">
         <v>261</v>
       </c>
@@ -10040,7 +10040,7 @@
         <v>2.3533050791148899E-8</v>
       </c>
     </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A186" s="27" t="s">
         <v>262</v>
       </c>
@@ -10078,7 +10078,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A187" s="27" t="s">
         <v>263</v>
       </c>
@@ -10116,7 +10116,7 @@
         <v>-0.187</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A188" s="27" t="s">
         <v>264</v>
       </c>
@@ -10154,7 +10154,7 @@
         <v>2.48</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A189" s="27" t="s">
         <v>265</v>
       </c>
@@ -10192,7 +10192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A190" s="27" t="s">
         <v>266</v>
       </c>
@@ -10230,7 +10230,7 @@
         <v>6.1060227588121015E-4</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A191" s="23" t="s">
         <v>267</v>
       </c>
@@ -10268,7 +10268,7 @@
         <v>3.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A192" s="23" t="s">
         <v>268</v>
       </c>
@@ -10306,7 +10306,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A193" s="23" t="s">
         <v>269</v>
       </c>
@@ -10344,7 +10344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A194" s="23" t="s">
         <v>270</v>
       </c>
@@ -10382,7 +10382,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="195" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A195" s="23" t="s">
         <v>271</v>
       </c>
@@ -10420,7 +10420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A196" s="23" t="s">
         <v>272</v>
       </c>
@@ -10458,7 +10458,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="197" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A197" s="7" t="s">
         <v>273</v>
       </c>
@@ -10496,7 +10496,7 @@
         <v>3.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="198" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A198" s="7" t="s">
         <v>274</v>
       </c>
@@ -10534,7 +10534,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="199" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A199" s="7" t="s">
         <v>275</v>
       </c>
@@ -10572,7 +10572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A200" s="7" t="s">
         <v>276</v>
       </c>
@@ -10610,7 +10610,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A201" s="7" t="s">
         <v>277</v>
       </c>
@@ -10648,7 +10648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A202" s="7" t="s">
         <v>278</v>
       </c>
@@ -10686,7 +10686,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A203" s="29" t="s">
         <v>279</v>
       </c>
@@ -10724,7 +10724,7 @@
         <v>1.9999999999999999E-7</v>
       </c>
     </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A204" s="29" t="s">
         <v>280</v>
       </c>
@@ -10762,7 +10762,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A205" s="29" t="s">
         <v>281</v>
       </c>
@@ -10800,7 +10800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A206" s="29" t="s">
         <v>282</v>
       </c>
@@ -10838,7 +10838,7 @@
         <v>3.98</v>
       </c>
     </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A207" s="29" t="s">
         <v>283</v>
       </c>
@@ -10876,7 +10876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A208" s="29" t="s">
         <v>284</v>
       </c>
@@ -10914,7 +10914,7 @@
         <v>8.3333333333333331E-5</v>
       </c>
     </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A209" s="90" t="s">
         <v>362</v>
       </c>
@@ -10952,7 +10952,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="210" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>569</v>
       </c>
@@ -10994,7 +10994,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="211" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>572</v>
       </c>
@@ -11033,7 +11033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>516</v>
       </c>
@@ -11060,11 +11060,10 @@
         <v>0.3</v>
       </c>
       <c r="I212" s="83">
-        <f t="shared" ref="I212:J212" si="4">I211</f>
-        <v>0.3</v>
+        <v>-10000</v>
       </c>
       <c r="J212" s="83">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I212:J212" si="4">J211</f>
         <v>0.3</v>
       </c>
       <c r="K212" s="1"/>
@@ -11075,7 +11074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>575</v>
       </c>
@@ -11116,7 +11115,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="214" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>508</v>
       </c>
@@ -11155,7 +11154,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="215" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>509</v>
       </c>
@@ -11194,7 +11193,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="216" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:13" s="96" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
         <v>510</v>
       </c>
@@ -11233,7 +11232,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>518</v>
       </c>
@@ -11271,7 +11270,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
         <v>520</v>
       </c>
@@ -11313,7 +11312,7 @@
         <v>2.5000000000000001E-4</v>
       </c>
     </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
         <v>523</v>
       </c>
@@ -11351,7 +11350,7 @@
         <v>9.9999999999999994E-12</v>
       </c>
     </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
         <v>526</v>
       </c>
@@ -11389,7 +11388,7 @@
         <v>2.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A221" s="2" t="s">
         <v>542</v>
       </c>
@@ -11421,7 +11420,7 @@
         <v>2.4999999999999999E-13</v>
       </c>
     </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>543</v>
       </c>
@@ -11456,7 +11455,7 @@
         <v>1.1999999999999999E-5</v>
       </c>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A223" s="2" t="s">
         <v>544</v>
       </c>
@@ -11488,7 +11487,7 @@
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A224" s="2" t="s">
         <v>545</v>
       </c>
@@ -11521,7 +11520,7 @@
         <v>5.0000000000000002E-5</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A225" s="2" t="s">
         <v>523</v>
       </c>
@@ -11557,7 +11556,7 @@
         <v>8.0000000000000003E-10</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A226" s="2" t="s">
         <v>546</v>
       </c>
@@ -11593,7 +11592,7 @@
         <v>8.0000000000000005E-9</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
         <v>547</v>
       </c>
@@ -11629,7 +11628,7 @@
         <v>0.10886399999999999</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
         <v>548</v>
       </c>
@@ -11661,7 +11660,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A229" s="2" t="s">
         <v>549</v>
       </c>
@@ -11693,7 +11692,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A230" s="2" t="s">
         <v>550</v>
       </c>
@@ -11729,7 +11728,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A231" s="2" t="s">
         <v>551</v>
       </c>
@@ -11761,7 +11760,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
         <v>552</v>
       </c>
@@ -11793,7 +11792,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A233" s="2" t="s">
         <v>578</v>
       </c>
@@ -11813,7 +11812,7 @@
         <v>571</v>
       </c>
       <c r="G233" s="83">
-        <f t="shared" ref="G233:J234" si="12">0.00002 / 14 / 5</f>
+        <f t="shared" ref="G233:J233" si="12">0.00002 / 14 / 5</f>
         <v>2.8571428571428575E-7</v>
       </c>
       <c r="H233" s="83">
@@ -11821,15 +11820,14 @@
         <v>2.8571428571428575E-7</v>
       </c>
       <c r="I233" s="83">
-        <f t="shared" si="12"/>
-        <v>2.8571428571428575E-7</v>
+        <v>0</v>
       </c>
       <c r="J233" s="83">
         <f t="shared" si="12"/>
         <v>2.8571428571428575E-7</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A234" s="2" t="s">
         <v>579</v>
       </c>
@@ -11857,8 +11855,7 @@
         <v>2.8571428571428575E-8</v>
       </c>
       <c r="I234" s="83">
-        <f>0.00002 / 14 / 5 /10</f>
-        <v>2.8571428571428575E-8</v>
+        <v>0</v>
       </c>
       <c r="J234" s="83">
         <f>0.00002 / 14 / 5 /10</f>
@@ -11866,8 +11863,216 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L127:M128">
-    <cfRule type="colorScale" priority="45">
+  <conditionalFormatting sqref="G233:I234">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G234:J234">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H127:J128">
+    <cfRule type="colorScale" priority="287">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H129:J129 L129:M129">
+    <cfRule type="colorScale" priority="289">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="290">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H130:J130 L130:M130">
+    <cfRule type="colorScale" priority="293">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="294">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H132:J132 L132:M132">
+    <cfRule type="colorScale" priority="297">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="298">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H133:J133 L133:M133">
+    <cfRule type="colorScale" priority="302">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="301">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H138:J138 L138:M138">
+    <cfRule type="colorScale" priority="305">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H144:J144 L144:M144">
+    <cfRule type="colorScale" priority="309">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="308">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="307">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H160:J160 L160:M160">
+    <cfRule type="colorScale" priority="315">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="314">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="313">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -11967,7 +12172,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H214:J214">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -11977,7 +12182,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="20">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -11989,7 +12194,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H215:J215">
-    <cfRule type="colorScale" priority="21">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -11999,7 +12204,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="22">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12011,16 +12216,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H216:J216">
-    <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
@@ -12031,205 +12226,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H127:J128">
-    <cfRule type="colorScale" priority="287">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H129:J129 L129:M129">
-    <cfRule type="colorScale" priority="289">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="290">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H130:J130 L130:M130">
-    <cfRule type="colorScale" priority="293">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="294">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H132:J132 L132:M132">
-    <cfRule type="colorScale" priority="297">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="298">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H133:J133 L133:M133">
-    <cfRule type="colorScale" priority="301">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="302">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H138:J138 L138:M138">
-    <cfRule type="colorScale" priority="305">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H144:J144 L144:M144">
-    <cfRule type="colorScale" priority="307">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="308">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="309">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H160:J160 L160:M160">
-    <cfRule type="colorScale" priority="313">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="314">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="315">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L166:M166 H166:J166">
-    <cfRule type="colorScale" priority="319">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="320">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="321">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12395,16 +12392,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H228:J232">
-    <cfRule type="colorScale" priority="353">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="354">
       <colorScale>
         <cfvo type="min"/>
@@ -12415,19 +12402,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G233:I234">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="10">
+    <cfRule type="colorScale" priority="353">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12439,6 +12414,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J233">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -12449,7 +12434,9 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="8">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L127:M128">
+    <cfRule type="colorScale" priority="45">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12460,8 +12447,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G234:J234">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="L166:M166 H166:J166">
+    <cfRule type="colorScale" priority="320">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12471,7 +12458,17 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="319">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="321">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -12490,13 +12487,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C169"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="35.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.5703125" customWidth="1"/>
+    <col min="1" max="2" width="35.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>286</v>
       </c>
@@ -12507,7 +12504,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>206</v>
       </c>
@@ -12519,7 +12516,7 @@
         <v>pi</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -12531,7 +12528,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -12543,7 +12540,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>207</v>
       </c>
@@ -12555,7 +12552,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -12567,7 +12564,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -12579,7 +12576,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -12591,7 +12588,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -12603,7 +12600,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -12615,7 +12612,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -12627,7 +12624,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -12639,7 +12636,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -12651,7 +12648,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -12663,7 +12660,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -12675,7 +12672,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>208</v>
       </c>
@@ -12687,7 +12684,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -12699,7 +12696,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -12711,7 +12708,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>205</v>
       </c>
@@ -12723,7 +12720,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -12735,7 +12732,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -12747,7 +12744,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -12759,7 +12756,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -12771,7 +12768,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -12783,7 +12780,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -12795,7 +12792,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>209</v>
       </c>
@@ -12807,7 +12804,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>210</v>
       </c>
@@ -12819,7 +12816,7 @@
         <v>root_growth_T_ref</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>211</v>
       </c>
@@ -12831,7 +12828,7 @@
         <v>root_growth_A</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>212</v>
       </c>
@@ -12843,7 +12840,7 @@
         <v>root_growth_B</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>213</v>
       </c>
@@ -12855,7 +12852,7 @@
         <v>root_growth_C</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>214</v>
       </c>
@@ -12867,7 +12864,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>215</v>
       </c>
@@ -12879,7 +12876,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>216</v>
       </c>
@@ -12891,7 +12888,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>217</v>
       </c>
@@ -12903,7 +12900,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>218</v>
       </c>
@@ -12915,7 +12912,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>61</v>
       </c>
@@ -12927,7 +12924,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -12939,7 +12936,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>219</v>
       </c>
@@ -12951,7 +12948,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>220</v>
       </c>
@@ -12963,7 +12960,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>221</v>
       </c>
@@ -12975,7 +12972,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>222</v>
       </c>
@@ -12987,7 +12984,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>76</v>
       </c>
@@ -12999,7 +12996,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>223</v>
       </c>
@@ -13011,7 +13008,7 @@
         <v>expected_C_sucrose_root</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>224</v>
       </c>
@@ -13023,7 +13020,7 @@
         <v>expected_C_hexose_root</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>225</v>
       </c>
@@ -13035,7 +13032,7 @@
         <v>expected_C_hexose_soil</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>226</v>
       </c>
@@ -13047,7 +13044,7 @@
         <v>expected_C_hexose_reserve</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>65</v>
       </c>
@@ -13059,7 +13056,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>77</v>
       </c>
@@ -13071,7 +13068,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>227</v>
       </c>
@@ -13083,7 +13080,7 @@
         <v>surfacic_unloading_rate_reference</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>228</v>
       </c>
@@ -13095,7 +13092,7 @@
         <v>surfacic_unloading_rate_primordium</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>66</v>
       </c>
@@ -13107,7 +13104,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>229</v>
       </c>
@@ -13119,7 +13116,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>230</v>
       </c>
@@ -13131,7 +13128,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>231</v>
       </c>
@@ -13143,7 +13140,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>232</v>
       </c>
@@ -13155,7 +13152,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -13167,7 +13164,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>233</v>
       </c>
@@ -13179,7 +13176,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>234</v>
       </c>
@@ -13191,7 +13188,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>235</v>
       </c>
@@ -13203,7 +13200,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>236</v>
       </c>
@@ -13215,7 +13212,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -13227,7 +13224,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -13239,7 +13236,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -13251,7 +13248,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -13263,7 +13260,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>56</v>
       </c>
@@ -13275,7 +13272,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>58</v>
       </c>
@@ -13287,7 +13284,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -13299,7 +13296,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>237</v>
       </c>
@@ -13311,7 +13308,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>238</v>
       </c>
@@ -13323,7 +13320,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>239</v>
       </c>
@@ -13335,7 +13332,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>240</v>
       </c>
@@ -13347,7 +13344,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -13359,7 +13356,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -13371,7 +13368,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>241</v>
       </c>
@@ -13383,7 +13380,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>242</v>
       </c>
@@ -13395,7 +13392,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>243</v>
       </c>
@@ -13407,7 +13404,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>244</v>
       </c>
@@ -13419,7 +13416,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>74</v>
       </c>
@@ -13431,7 +13428,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>245</v>
       </c>
@@ -13443,7 +13440,7 @@
         <v>expected_exudation_efflux</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -13455,7 +13452,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>246</v>
       </c>
@@ -13467,7 +13464,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>247</v>
       </c>
@@ -13479,7 +13476,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>248</v>
       </c>
@@ -13491,7 +13488,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>249</v>
       </c>
@@ -13503,7 +13500,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -13515,7 +13512,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>80</v>
       </c>
@@ -13527,7 +13524,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>250</v>
       </c>
@@ -13539,7 +13536,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>251</v>
       </c>
@@ -13551,7 +13548,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>252</v>
       </c>
@@ -13563,7 +13560,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>253</v>
       </c>
@@ -13575,7 +13572,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>81</v>
       </c>
@@ -13587,7 +13584,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>254</v>
       </c>
@@ -13599,7 +13596,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>255</v>
       </c>
@@ -13611,7 +13608,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>256</v>
       </c>
@@ -13623,7 +13620,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>257</v>
       </c>
@@ -13635,7 +13632,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>258</v>
       </c>
@@ -13647,7 +13644,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>259</v>
       </c>
@@ -13659,7 +13656,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>260</v>
       </c>
@@ -13671,7 +13668,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>261</v>
       </c>
@@ -13683,7 +13680,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>262</v>
       </c>
@@ -13695,7 +13692,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>263</v>
       </c>
@@ -13707,7 +13704,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>264</v>
       </c>
@@ -13719,7 +13716,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>265</v>
       </c>
@@ -13731,7 +13728,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>266</v>
       </c>
@@ -13743,7 +13740,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>267</v>
       </c>
@@ -13755,7 +13752,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>268</v>
       </c>
@@ -13767,7 +13764,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>269</v>
       </c>
@@ -13779,7 +13776,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>270</v>
       </c>
@@ -13791,7 +13788,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>271</v>
       </c>
@@ -13803,7 +13800,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>272</v>
       </c>
@@ -13815,7 +13812,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>273</v>
       </c>
@@ -13827,7 +13824,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>274</v>
       </c>
@@ -13839,7 +13836,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>275</v>
       </c>
@@ -13851,7 +13848,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>276</v>
       </c>
@@ -13863,7 +13860,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>277</v>
       </c>
@@ -13875,7 +13872,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>278</v>
       </c>
@@ -13887,7 +13884,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>279</v>
       </c>
@@ -13899,7 +13896,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>280</v>
       </c>
@@ -13911,7 +13908,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>281</v>
       </c>
@@ -13923,7 +13920,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>282</v>
       </c>
@@ -13935,7 +13932,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>283</v>
       </c>
@@ -13947,7 +13944,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>284</v>
       </c>
@@ -13959,7 +13956,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>59</v>
       </c>
@@ -13971,7 +13968,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>62</v>
       </c>
@@ -13983,7 +13980,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>64</v>
       </c>
@@ -13995,7 +13992,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>63</v>
       </c>
@@ -14007,7 +14004,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>82</v>
       </c>
@@ -14019,7 +14016,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>83</v>
       </c>
@@ -14031,7 +14028,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>85</v>
       </c>
@@ -14043,7 +14040,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>84</v>
       </c>
@@ -14055,7 +14052,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>2</v>
       </c>
@@ -14067,7 +14064,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>4</v>
       </c>
@@ -14079,7 +14076,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>5</v>
       </c>
@@ -14091,7 +14088,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>20</v>
       </c>
@@ -14103,7 +14100,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>0</v>
       </c>
@@ -14115,7 +14112,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>1</v>
       </c>
@@ -14127,7 +14124,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>6</v>
       </c>
@@ -14139,7 +14136,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>7</v>
       </c>
@@ -14151,7 +14148,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -14163,7 +14160,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>9</v>
       </c>
@@ -14175,7 +14172,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>10</v>
       </c>
@@ -14187,7 +14184,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>11</v>
       </c>
@@ -14199,7 +14196,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>12</v>
       </c>
@@ -14211,7 +14208,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -14223,7 +14220,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>14</v>
       </c>
@@ -14235,7 +14232,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>15</v>
       </c>
@@ -14247,7 +14244,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -14259,7 +14256,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>17</v>
       </c>
@@ -14271,7 +14268,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>18</v>
       </c>
@@ -14283,7 +14280,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>19</v>
       </c>
@@ -14295,7 +14292,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -14307,7 +14304,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>22</v>
       </c>
@@ -14319,7 +14316,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>23</v>
       </c>
@@ -14331,7 +14328,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>24</v>
       </c>
@@ -14343,7 +14340,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>25</v>
       </c>
@@ -14355,7 +14352,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>26</v>
       </c>
@@ -14367,7 +14364,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>27</v>
       </c>
@@ -14379,7 +14376,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>28</v>
       </c>
@@ -14388,7 +14385,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>29</v>
       </c>
@@ -14397,7 +14394,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -14406,7 +14403,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>31</v>
       </c>
@@ -14415,7 +14412,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>32</v>
       </c>
@@ -14424,7 +14421,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>33</v>
       </c>
@@ -14433,7 +14430,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>34</v>
       </c>
@@ -14442,7 +14439,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>35</v>
       </c>
@@ -14451,7 +14448,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>36</v>
       </c>
@@ -14460,7 +14457,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>37</v>
       </c>
@@ -14469,7 +14466,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>38</v>
       </c>
@@ -14478,7 +14475,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>362</v>
       </c>

</xml_diff>

<commit_message>
removed reference to families
</commit_message>
<xml_diff>
--- a/simulations/inputs/Scenarios_24_11_10.xlsx
+++ b/simulations/inputs/Scenarios_24_11_10.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp16152\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp31710\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8297F2DF-1CD3-49A1-B936-DC158CBDEFE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB0F955-655A-409C-BE0D-A74A90ED9A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25320" yWindow="-15990" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios_as_columns" sheetId="2" r:id="rId1"/>
@@ -14912,8 +14912,7 @@
         <v>2.8571428571428575E-8</v>
       </c>
       <c r="L233" s="83">
-        <f t="shared" si="24"/>
-        <v>2.8571428571428575E-8</v>
+        <v>0</v>
       </c>
       <c r="M233" s="83">
         <f t="shared" si="24"/>
@@ -14921,7 +14920,7 @@
       </c>
       <c r="O233" s="1" t="b">
         <f t="shared" si="17"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -14982,7 +14981,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H210:M210">
-    <cfRule type="colorScale" priority="364">
+    <cfRule type="colorScale" priority="365">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14992,7 +14991,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="365">
+    <cfRule type="colorScale" priority="364">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15004,7 +15003,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H211:M211">
-    <cfRule type="colorScale" priority="366">
+    <cfRule type="colorScale" priority="367">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15014,7 +15013,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="367">
+    <cfRule type="colorScale" priority="366">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15048,7 +15047,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H213:M213">
-    <cfRule type="colorScale" priority="370">
+    <cfRule type="colorScale" priority="371">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15058,7 +15057,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="371">
+    <cfRule type="colorScale" priority="370">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15070,7 +15069,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H214:M214">
-    <cfRule type="colorScale" priority="372">
+    <cfRule type="colorScale" priority="373">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15080,7 +15079,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="373">
+    <cfRule type="colorScale" priority="372">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15092,7 +15091,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H215:M215">
-    <cfRule type="colorScale" priority="374">
+    <cfRule type="colorScale" priority="375">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15102,7 +15101,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="375">
+    <cfRule type="colorScale" priority="374">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15114,7 +15113,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H218:M218">
-    <cfRule type="colorScale" priority="376">
+    <cfRule type="colorScale" priority="377">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15124,7 +15123,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="377">
+    <cfRule type="colorScale" priority="376">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15136,7 +15135,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H219:M221">
-    <cfRule type="colorScale" priority="390">
+    <cfRule type="colorScale" priority="391">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15146,7 +15145,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="391">
+    <cfRule type="colorScale" priority="390">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15158,7 +15157,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H222:M222">
-    <cfRule type="colorScale" priority="380">
+    <cfRule type="colorScale" priority="381">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15168,7 +15167,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="381">
+    <cfRule type="colorScale" priority="380">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15180,7 +15179,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H226:M226">
-    <cfRule type="colorScale" priority="384">
+    <cfRule type="colorScale" priority="385">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15190,7 +15189,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="385">
+    <cfRule type="colorScale" priority="384">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15224,16 +15223,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H223:N223 H224:M224">
-    <cfRule type="colorScale" priority="382">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="383">
       <colorScale>
         <cfvo type="min"/>
@@ -15244,19 +15233,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P132:Q132 H132:N132">
-    <cfRule type="colorScale" priority="303">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="304">
+    <cfRule type="colorScale" priority="382">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15290,7 +15267,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K232:K233">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15300,7 +15277,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15389,8 +15366,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P133:Q133 H133:M133">
-    <cfRule type="colorScale" priority="307">
+  <conditionalFormatting sqref="P132:Q132 H132:N132">
+    <cfRule type="colorScale" priority="304">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15400,7 +15377,29 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="303">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P133:Q133 H133:M133">
     <cfRule type="colorScale" priority="308">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="307">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15456,6 +15455,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P160:Q160 H160:M160">
+    <cfRule type="colorScale" priority="321">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="319">
       <colorScale>
         <cfvo type="min"/>
@@ -15476,7 +15485,9 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="321">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P166:Q166 H166:M166">
+    <cfRule type="colorScale" priority="326">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15486,19 +15497,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P166:Q166 H166:M166">
     <cfRule type="colorScale" priority="325">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="326">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>